<commit_message>
feat: simplifica situações dos itens para quatro opções e ajusta cursores
Situações passam a ser Pesquisando, Comprado, Recebido e Já tenho; as antigas
migram para Pesquisando. Remove cursores customizados e os cursores grab.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/modelos/casamia-modelo-importacao.xlsx
+++ b/public/modelos/casamia-modelo-importacao.xlsx
@@ -47,7 +47,7 @@
     <t>Quarto</t>
   </si>
   <si>
-    <t>Comprei</t>
+    <t>Comprado</t>
   </si>
   <si>
     <t>https://www.exemplo.com.br/jogo-de-cama</t>
@@ -59,15 +59,12 @@
     <t>Travesseiro de plumas</t>
   </si>
   <si>
-    <t>Preciso comprar</t>
+    <t>Pesquisando</t>
   </si>
   <si>
     <t>Cortina blackout</t>
   </si>
   <si>
-    <t>Pesquisando</t>
-  </si>
-  <si>
     <t>Comparar tamanhos de 2,20 m</t>
   </si>
   <si>
@@ -77,7 +74,7 @@
     <t>Banheiro</t>
   </si>
   <si>
-    <t>Ganhei</t>
+    <t>Recebido</t>
   </si>
   <si>
     <t>Presente da tia Marta</t>
@@ -116,10 +113,7 @@
     <t>Sala de Estar</t>
   </si>
   <si>
-    <t>Mesa de jantar (não preciso mais)</t>
-  </si>
-  <si>
-    <t>Não preciso</t>
+    <t>Mesa de jantar</t>
   </si>
   <si>
     <t>Já ganhamos uma</t>
@@ -146,7 +140,7 @@
     <t>Onde o item fica (Quarto, Cozinha...). Ambientes que ainda não existem são criados. Até 24 caracteres.</t>
   </si>
   <si>
-    <t>Preciso comprar · Pesquisando · Comprei · Ganhei · Já tenho · Não preciso · Descartei. Em branco = Preciso comprar.</t>
+    <t>Pesquisando · Comprado · Recebido · Já tenho. Em branco = Pesquisando.</t>
   </si>
   <si>
     <t>Não</t>
@@ -158,7 +152,7 @@
     <t>Valor do item, como 249,90 ou 1.249,90. Em branco = sem preço.</t>
   </si>
   <si>
-    <t>Só vale para Preciso comprar, Pesquisando e Comprei, e precisa ser menor ou igual ao preço.</t>
+    <t>Só vale para Pesquisando e Comprado, e precisa ser menor ou igual ao preço.</t>
   </si>
   <si>
     <t>Endereço da loja ou do produto.</t>
@@ -332,24 +326,24 @@
         <v>9</v>
       </c>
       <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
         <v>16</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="H4" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>19</v>
-      </c>
-      <c r="C5" t="s">
-        <v>20</v>
       </c>
       <c r="D5">
         <v>4</v>
@@ -358,18 +352,18 @@
         <v>120</v>
       </c>
       <c r="H5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
         <v>22</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" t="s">
-        <v>23</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -377,10 +371,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
         <v>24</v>
-      </c>
-      <c r="B7" t="s">
-        <v>25</v>
       </c>
       <c r="C7" t="s">
         <v>14</v>
@@ -392,18 +386,18 @@
         <v>3499</v>
       </c>
       <c r="G7" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" t="s">
         <v>26</v>
-      </c>
-      <c r="H7" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
         <v>10</v>
@@ -417,10 +411,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
         <v>29</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
       </c>
       <c r="C9" t="s">
         <v>14</v>
@@ -434,13 +428,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s">
         <v>31</v>
       </c>
-      <c r="B10" t="s">
-        <v>32</v>
-      </c>
       <c r="C10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -451,19 +445,19 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="H11" t="s">
         <v>33</v>
-      </c>
-      <c r="B11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="H11" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -480,7 +474,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
@@ -488,13 +482,13 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="4">
@@ -502,10 +496,10 @@
         <v>0</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -513,10 +507,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -524,10 +518,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7">
@@ -535,10 +529,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -546,10 +540,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
@@ -557,10 +551,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10">
@@ -568,10 +562,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11">
@@ -579,10 +573,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12">
@@ -590,32 +584,32 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Meu enxoval com mais valor (parcelas, responsável, presentes, comprovantes, lojas, modo loja) e formulário de item unificado
</commit_message>
<xml_diff>
--- a/public/modelos/casamia-modelo-importacao.xlsx
+++ b/public/modelos/casamia-modelo-importacao.xlsx
@@ -137,7 +137,10 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>Onde o item fica (Quarto, Cozinha...). Ambientes que ainda não existem são criados. Até 24 caracteres.</t>
+    <t>Onde o item fica (Quarto, Cozinha...). Ambientes que ainda não existem são criados. Até 24 caracteres. Em branco: o catálogo sugere o ambiente dos itens que conhece.</t>
+  </si>
+  <si>
+    <t>Sim, salvo itens que o catálogo conhece</t>
   </si>
   <si>
     <t>Pesquisando · Comprado · Recebido · Já tenho. Em branco = Pesquisando.</t>
@@ -164,7 +167,7 @@
     <t>Dicas</t>
   </si>
   <si>
-    <t>Item e Ambiente são obrigatórios e precisam estar preenchidos em todas as linhas. Se faltar algo, o arquivo é recusado e nada é importado.</t>
+    <t>Item é obrigatório em todas as linhas, e Ambiente também, a não ser que o catálogo conheça o item. Se faltar algo, o arquivo é recusado e nada é importado.</t>
   </si>
   <si>
     <t>A primeira linha da aba "Itens" deve manter os títulos das colunas.</t>
@@ -510,7 +513,7 @@
         <v>40</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6">
@@ -518,10 +521,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
@@ -529,10 +532,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -540,10 +543,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9">
@@ -551,10 +554,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10">
@@ -562,10 +565,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11">
@@ -573,10 +576,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12">
@@ -584,32 +587,32 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>